<commit_message>
some changes in loginsteps
</commit_message>
<xml_diff>
--- a/MCP_Reports_Pro/src/test/resources/testdata/LoginData.xlsx
+++ b/MCP_Reports_Pro/src/test/resources/testdata/LoginData.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\harsh\IdeaProjects\MCP_Reports_Pro\src\test\resources\testdata\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Jenkins\MCP_Reports_Pro\src\test\resources\testdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{06B33C35-8F30-4737-91BD-FC4F112A85E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{31B9F04E-F5F0-48A7-BB96-F3711C1EA1AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{51D5159A-F34C-4423-8842-29BA0F49478D}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="9">
   <si>
     <t>Username</t>
   </si>
@@ -58,6 +58,9 @@
   </si>
   <si>
     <t>Test@123</t>
+  </si>
+  <si>
+    <t>fail</t>
   </si>
 </sst>
 </file>
@@ -541,7 +544,7 @@
         <v>6</v>
       </c>
       <c r="C10" t="s">
-        <v>3</v>
+        <v>8</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.3">
@@ -552,7 +555,7 @@
         <v>6</v>
       </c>
       <c r="C11" t="s">
-        <v>3</v>
+        <v>8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>